<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@e064be8ebe5c002865cdd8182dad9010a8bc4936 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-AllergyIntolerance.xlsx
+++ b/StructureDefinition-AllergyIntolerance.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AQ$185</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AQ$189</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7234" uniqueCount="689">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7391" uniqueCount="693">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-07-26T12:02:04+00:00</t>
+    <t>2024-07-26T12:19:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2010,6 +2010,18 @@
   </si>
   <si>
     <t>AL1-5</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.reaction.manifestation.id</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.reaction.manifestation.extension</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.reaction.manifestation.coding</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.reaction.manifestation.text</t>
   </si>
   <si>
     <t>AllergyIntolerance.reaction.description</t>
@@ -2492,7 +2504,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AQ185"/>
+  <dimension ref="A1:AQ189"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="92.64453125" customWidth="true" bestFit="true"/>
@@ -6589,7 +6601,7 @@
         <v>90</v>
       </c>
       <c r="H34" t="s" s="2">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="I34" t="s" s="2">
         <v>81</v>
@@ -23450,7 +23462,7 @@
         <v>80</v>
       </c>
       <c r="H171" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="I171" t="s" s="2">
         <v>81</v>
@@ -23561,7 +23573,7 @@
       </c>
       <c r="C172" s="2"/>
       <c r="D172" t="s" s="2">
-        <v>639</v>
+        <v>81</v>
       </c>
       <c r="E172" s="2"/>
       <c r="F172" t="s" s="2">
@@ -23583,14 +23595,12 @@
         <v>165</v>
       </c>
       <c r="L172" t="s" s="2">
-        <v>640</v>
+        <v>166</v>
       </c>
       <c r="M172" t="s" s="2">
-        <v>641</v>
-      </c>
-      <c r="N172" t="s" s="2">
-        <v>642</v>
-      </c>
+        <v>184</v>
+      </c>
+      <c r="N172" s="2"/>
       <c r="O172" s="2"/>
       <c r="P172" t="s" s="2">
         <v>81</v>
@@ -23639,7 +23649,7 @@
         <v>81</v>
       </c>
       <c r="AF172" t="s" s="2">
-        <v>638</v>
+        <v>168</v>
       </c>
       <c r="AG172" t="s" s="2">
         <v>79</v>
@@ -23654,19 +23664,19 @@
         <v>81</v>
       </c>
       <c r="AK172" t="s" s="2">
-        <v>643</v>
+        <v>81</v>
       </c>
       <c r="AL172" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM172" t="s" s="2">
-        <v>643</v>
+        <v>81</v>
       </c>
       <c r="AN172" t="s" s="2">
-        <v>643</v>
+        <v>81</v>
       </c>
       <c r="AO172" t="s" s="2">
-        <v>644</v>
+        <v>185</v>
       </c>
       <c r="AP172" t="s" s="2">
         <v>81</v>
@@ -23677,21 +23687,21 @@
     </row>
     <row r="173" hidden="true">
       <c r="A173" t="s" s="2">
-        <v>645</v>
+        <v>639</v>
       </c>
       <c r="B173" t="s" s="2">
-        <v>645</v>
+        <v>639</v>
       </c>
       <c r="C173" s="2"/>
       <c r="D173" t="s" s="2">
-        <v>646</v>
+        <v>135</v>
       </c>
       <c r="E173" s="2"/>
       <c r="F173" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G173" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H173" t="s" s="2">
         <v>81</v>
@@ -23703,15 +23713,17 @@
         <v>81</v>
       </c>
       <c r="K173" t="s" s="2">
-        <v>432</v>
+        <v>136</v>
       </c>
       <c r="L173" t="s" s="2">
-        <v>647</v>
+        <v>137</v>
       </c>
       <c r="M173" t="s" s="2">
-        <v>648</v>
-      </c>
-      <c r="N173" s="2"/>
+        <v>188</v>
+      </c>
+      <c r="N173" t="s" s="2">
+        <v>139</v>
+      </c>
       <c r="O173" s="2"/>
       <c r="P173" t="s" s="2">
         <v>81</v>
@@ -23748,25 +23760,25 @@
         <v>81</v>
       </c>
       <c r="AB173" t="s" s="2">
-        <v>81</v>
+        <v>172</v>
       </c>
       <c r="AC173" t="s" s="2">
-        <v>81</v>
+        <v>189</v>
       </c>
       <c r="AD173" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE173" t="s" s="2">
-        <v>81</v>
+        <v>173</v>
       </c>
       <c r="AF173" t="s" s="2">
-        <v>645</v>
+        <v>174</v>
       </c>
       <c r="AG173" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH173" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AI173" t="s" s="2">
         <v>81</v>
@@ -23775,44 +23787,44 @@
         <v>81</v>
       </c>
       <c r="AK173" t="s" s="2">
-        <v>649</v>
+        <v>81</v>
       </c>
       <c r="AL173" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM173" t="s" s="2">
-        <v>649</v>
+        <v>81</v>
       </c>
       <c r="AN173" t="s" s="2">
-        <v>649</v>
+        <v>81</v>
       </c>
       <c r="AO173" t="s" s="2">
-        <v>427</v>
+        <v>185</v>
       </c>
       <c r="AP173" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AQ173" t="s" s="2">
-        <v>650</v>
+        <v>81</v>
       </c>
     </row>
     <row r="174" hidden="true">
       <c r="A174" t="s" s="2">
-        <v>651</v>
+        <v>640</v>
       </c>
       <c r="B174" t="s" s="2">
-        <v>651</v>
+        <v>640</v>
       </c>
       <c r="C174" s="2"/>
       <c r="D174" t="s" s="2">
-        <v>652</v>
+        <v>81</v>
       </c>
       <c r="E174" s="2"/>
       <c r="F174" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G174" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H174" t="s" s="2">
         <v>81</v>
@@ -23821,21 +23833,23 @@
         <v>81</v>
       </c>
       <c r="J174" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="K174" t="s" s="2">
-        <v>109</v>
+        <v>297</v>
       </c>
       <c r="L174" t="s" s="2">
-        <v>653</v>
+        <v>298</v>
       </c>
       <c r="M174" t="s" s="2">
-        <v>654</v>
+        <v>299</v>
       </c>
       <c r="N174" t="s" s="2">
-        <v>655</v>
-      </c>
-      <c r="O174" s="2"/>
+        <v>300</v>
+      </c>
+      <c r="O174" t="s" s="2">
+        <v>301</v>
+      </c>
       <c r="P174" t="s" s="2">
         <v>81</v>
       </c>
@@ -23859,11 +23873,13 @@
         <v>81</v>
       </c>
       <c r="X174" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="Y174" s="2"/>
+        <v>81</v>
+      </c>
+      <c r="Y174" t="s" s="2">
+        <v>81</v>
+      </c>
       <c r="Z174" t="s" s="2">
-        <v>656</v>
+        <v>81</v>
       </c>
       <c r="AA174" t="s" s="2">
         <v>81</v>
@@ -23881,13 +23897,13 @@
         <v>81</v>
       </c>
       <c r="AF174" t="s" s="2">
-        <v>651</v>
+        <v>303</v>
       </c>
       <c r="AG174" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH174" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AI174" t="s" s="2">
         <v>81</v>
@@ -23896,33 +23912,33 @@
         <v>81</v>
       </c>
       <c r="AK174" t="s" s="2">
-        <v>657</v>
+        <v>81</v>
       </c>
       <c r="AL174" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM174" t="s" s="2">
-        <v>657</v>
+        <v>81</v>
       </c>
       <c r="AN174" t="s" s="2">
-        <v>657</v>
+        <v>81</v>
       </c>
       <c r="AO174" t="s" s="2">
-        <v>260</v>
+        <v>304</v>
       </c>
       <c r="AP174" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AQ174" t="s" s="2">
-        <v>81</v>
+        <v>305</v>
       </c>
     </row>
     <row r="175" hidden="true">
       <c r="A175" t="s" s="2">
-        <v>658</v>
+        <v>641</v>
       </c>
       <c r="B175" t="s" s="2">
-        <v>658</v>
+        <v>641</v>
       </c>
       <c r="C175" s="2"/>
       <c r="D175" t="s" s="2">
@@ -23936,25 +23952,29 @@
         <v>90</v>
       </c>
       <c r="H175" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="I175" t="s" s="2">
         <v>81</v>
       </c>
       <c r="J175" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="K175" t="s" s="2">
         <v>165</v>
       </c>
       <c r="L175" t="s" s="2">
-        <v>166</v>
+        <v>407</v>
       </c>
       <c r="M175" t="s" s="2">
-        <v>167</v>
-      </c>
-      <c r="N175" s="2"/>
-      <c r="O175" s="2"/>
+        <v>408</v>
+      </c>
+      <c r="N175" t="s" s="2">
+        <v>409</v>
+      </c>
+      <c r="O175" t="s" s="2">
+        <v>410</v>
+      </c>
       <c r="P175" t="s" s="2">
         <v>81</v>
       </c>
@@ -24002,7 +24022,7 @@
         <v>81</v>
       </c>
       <c r="AF175" t="s" s="2">
-        <v>168</v>
+        <v>411</v>
       </c>
       <c r="AG175" t="s" s="2">
         <v>79</v>
@@ -24029,32 +24049,32 @@
         <v>81</v>
       </c>
       <c r="AO175" t="s" s="2">
-        <v>81</v>
+        <v>412</v>
       </c>
       <c r="AP175" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AQ175" t="s" s="2">
-        <v>81</v>
+        <v>413</v>
       </c>
     </row>
     <row r="176" hidden="true">
       <c r="A176" t="s" s="2">
-        <v>659</v>
+        <v>642</v>
       </c>
       <c r="B176" t="s" s="2">
-        <v>659</v>
+        <v>642</v>
       </c>
       <c r="C176" s="2"/>
       <c r="D176" t="s" s="2">
-        <v>81</v>
+        <v>643</v>
       </c>
       <c r="E176" s="2"/>
       <c r="F176" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G176" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H176" t="s" s="2">
         <v>81</v>
@@ -24066,15 +24086,17 @@
         <v>81</v>
       </c>
       <c r="K176" t="s" s="2">
-        <v>136</v>
+        <v>165</v>
       </c>
       <c r="L176" t="s" s="2">
-        <v>170</v>
+        <v>644</v>
       </c>
       <c r="M176" t="s" s="2">
-        <v>171</v>
-      </c>
-      <c r="N176" s="2"/>
+        <v>645</v>
+      </c>
+      <c r="N176" t="s" s="2">
+        <v>646</v>
+      </c>
       <c r="O176" s="2"/>
       <c r="P176" t="s" s="2">
         <v>81</v>
@@ -24111,23 +24133,25 @@
         <v>81</v>
       </c>
       <c r="AB176" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="AC176" s="2"/>
+        <v>81</v>
+      </c>
+      <c r="AC176" t="s" s="2">
+        <v>81</v>
+      </c>
       <c r="AD176" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE176" t="s" s="2">
-        <v>173</v>
+        <v>81</v>
       </c>
       <c r="AF176" t="s" s="2">
-        <v>174</v>
+        <v>642</v>
       </c>
       <c r="AG176" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH176" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AI176" t="s" s="2">
         <v>81</v>
@@ -24136,19 +24160,19 @@
         <v>81</v>
       </c>
       <c r="AK176" t="s" s="2">
-        <v>81</v>
+        <v>647</v>
       </c>
       <c r="AL176" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM176" t="s" s="2">
-        <v>81</v>
+        <v>647</v>
       </c>
       <c r="AN176" t="s" s="2">
-        <v>81</v>
+        <v>647</v>
       </c>
       <c r="AO176" t="s" s="2">
-        <v>81</v>
+        <v>648</v>
       </c>
       <c r="AP176" t="s" s="2">
         <v>81</v>
@@ -24159,23 +24183,21 @@
     </row>
     <row r="177" hidden="true">
       <c r="A177" t="s" s="2">
-        <v>660</v>
+        <v>649</v>
       </c>
       <c r="B177" t="s" s="2">
-        <v>659</v>
-      </c>
-      <c r="C177" t="s" s="2">
-        <v>661</v>
-      </c>
+        <v>649</v>
+      </c>
+      <c r="C177" s="2"/>
       <c r="D177" t="s" s="2">
-        <v>662</v>
+        <v>650</v>
       </c>
       <c r="E177" s="2"/>
       <c r="F177" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G177" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H177" t="s" s="2">
         <v>81</v>
@@ -24187,13 +24209,13 @@
         <v>81</v>
       </c>
       <c r="K177" t="s" s="2">
-        <v>178</v>
+        <v>432</v>
       </c>
       <c r="L177" t="s" s="2">
-        <v>663</v>
+        <v>651</v>
       </c>
       <c r="M177" t="s" s="2">
-        <v>664</v>
+        <v>652</v>
       </c>
       <c r="N177" s="2"/>
       <c r="O177" s="2"/>
@@ -24244,52 +24266,52 @@
         <v>81</v>
       </c>
       <c r="AF177" t="s" s="2">
-        <v>174</v>
+        <v>649</v>
       </c>
       <c r="AG177" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH177" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AI177" t="s" s="2">
-        <v>180</v>
+        <v>81</v>
       </c>
       <c r="AJ177" t="s" s="2">
-        <v>181</v>
+        <v>81</v>
       </c>
       <c r="AK177" t="s" s="2">
-        <v>81</v>
+        <v>653</v>
       </c>
       <c r="AL177" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM177" t="s" s="2">
-        <v>81</v>
+        <v>653</v>
       </c>
       <c r="AN177" t="s" s="2">
-        <v>81</v>
+        <v>653</v>
       </c>
       <c r="AO177" t="s" s="2">
-        <v>81</v>
+        <v>427</v>
       </c>
       <c r="AP177" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AQ177" t="s" s="2">
-        <v>81</v>
+        <v>654</v>
       </c>
     </row>
     <row r="178" hidden="true">
       <c r="A178" t="s" s="2">
-        <v>665</v>
+        <v>655</v>
       </c>
       <c r="B178" t="s" s="2">
-        <v>666</v>
+        <v>655</v>
       </c>
       <c r="C178" s="2"/>
       <c r="D178" t="s" s="2">
-        <v>81</v>
+        <v>656</v>
       </c>
       <c r="E178" s="2"/>
       <c r="F178" t="s" s="2">
@@ -24299,7 +24321,7 @@
         <v>90</v>
       </c>
       <c r="H178" t="s" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="I178" t="s" s="2">
         <v>81</v>
@@ -24308,15 +24330,17 @@
         <v>81</v>
       </c>
       <c r="K178" t="s" s="2">
-        <v>165</v>
+        <v>109</v>
       </c>
       <c r="L178" t="s" s="2">
-        <v>166</v>
+        <v>657</v>
       </c>
       <c r="M178" t="s" s="2">
-        <v>184</v>
-      </c>
-      <c r="N178" s="2"/>
+        <v>658</v>
+      </c>
+      <c r="N178" t="s" s="2">
+        <v>659</v>
+      </c>
       <c r="O178" s="2"/>
       <c r="P178" t="s" s="2">
         <v>81</v>
@@ -24341,13 +24365,11 @@
         <v>81</v>
       </c>
       <c r="X178" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="Y178" t="s" s="2">
-        <v>81</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="Y178" s="2"/>
       <c r="Z178" t="s" s="2">
-        <v>81</v>
+        <v>660</v>
       </c>
       <c r="AA178" t="s" s="2">
         <v>81</v>
@@ -24365,7 +24387,7 @@
         <v>81</v>
       </c>
       <c r="AF178" t="s" s="2">
-        <v>168</v>
+        <v>655</v>
       </c>
       <c r="AG178" t="s" s="2">
         <v>79</v>
@@ -24380,19 +24402,19 @@
         <v>81</v>
       </c>
       <c r="AK178" t="s" s="2">
-        <v>81</v>
+        <v>661</v>
       </c>
       <c r="AL178" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM178" t="s" s="2">
-        <v>81</v>
+        <v>661</v>
       </c>
       <c r="AN178" t="s" s="2">
-        <v>81</v>
+        <v>661</v>
       </c>
       <c r="AO178" t="s" s="2">
-        <v>185</v>
+        <v>260</v>
       </c>
       <c r="AP178" t="s" s="2">
         <v>81</v>
@@ -24403,21 +24425,21 @@
     </row>
     <row r="179" hidden="true">
       <c r="A179" t="s" s="2">
-        <v>667</v>
+        <v>662</v>
       </c>
       <c r="B179" t="s" s="2">
-        <v>668</v>
+        <v>662</v>
       </c>
       <c r="C179" s="2"/>
       <c r="D179" t="s" s="2">
-        <v>135</v>
+        <v>81</v>
       </c>
       <c r="E179" s="2"/>
       <c r="F179" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G179" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H179" t="s" s="2">
         <v>81</v>
@@ -24429,17 +24451,15 @@
         <v>81</v>
       </c>
       <c r="K179" t="s" s="2">
-        <v>136</v>
+        <v>165</v>
       </c>
       <c r="L179" t="s" s="2">
-        <v>137</v>
+        <v>166</v>
       </c>
       <c r="M179" t="s" s="2">
-        <v>188</v>
-      </c>
-      <c r="N179" t="s" s="2">
-        <v>139</v>
-      </c>
+        <v>167</v>
+      </c>
+      <c r="N179" s="2"/>
       <c r="O179" s="2"/>
       <c r="P179" t="s" s="2">
         <v>81</v>
@@ -24476,25 +24496,25 @@
         <v>81</v>
       </c>
       <c r="AB179" t="s" s="2">
-        <v>172</v>
+        <v>81</v>
       </c>
       <c r="AC179" t="s" s="2">
-        <v>189</v>
+        <v>81</v>
       </c>
       <c r="AD179" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE179" t="s" s="2">
-        <v>173</v>
+        <v>81</v>
       </c>
       <c r="AF179" t="s" s="2">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="AG179" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH179" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="AI179" t="s" s="2">
         <v>81</v>
@@ -24515,7 +24535,7 @@
         <v>81</v>
       </c>
       <c r="AO179" t="s" s="2">
-        <v>185</v>
+        <v>81</v>
       </c>
       <c r="AP179" t="s" s="2">
         <v>81</v>
@@ -24526,10 +24546,10 @@
     </row>
     <row r="180" hidden="true">
       <c r="A180" t="s" s="2">
-        <v>669</v>
+        <v>663</v>
       </c>
       <c r="B180" t="s" s="2">
-        <v>670</v>
+        <v>663</v>
       </c>
       <c r="C180" s="2"/>
       <c r="D180" t="s" s="2">
@@ -24537,10 +24557,10 @@
       </c>
       <c r="E180" s="2"/>
       <c r="F180" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="G180" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H180" t="s" s="2">
         <v>81</v>
@@ -24552,24 +24572,22 @@
         <v>81</v>
       </c>
       <c r="K180" t="s" s="2">
-        <v>103</v>
+        <v>136</v>
       </c>
       <c r="L180" t="s" s="2">
-        <v>192</v>
+        <v>170</v>
       </c>
       <c r="M180" t="s" s="2">
-        <v>193</v>
-      </c>
-      <c r="N180" t="s" s="2">
-        <v>194</v>
-      </c>
+        <v>171</v>
+      </c>
+      <c r="N180" s="2"/>
       <c r="O180" s="2"/>
       <c r="P180" t="s" s="2">
         <v>81</v>
       </c>
       <c r="Q180" s="2"/>
       <c r="R180" t="s" s="2">
-        <v>195</v>
+        <v>81</v>
       </c>
       <c r="S180" t="s" s="2">
         <v>81</v>
@@ -24599,25 +24617,23 @@
         <v>81</v>
       </c>
       <c r="AB180" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC180" t="s" s="2">
-        <v>81</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="AC180" s="2"/>
       <c r="AD180" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE180" t="s" s="2">
-        <v>81</v>
+        <v>173</v>
       </c>
       <c r="AF180" t="s" s="2">
-        <v>196</v>
+        <v>174</v>
       </c>
       <c r="AG180" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="AH180" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AI180" t="s" s="2">
         <v>81</v>
@@ -24638,7 +24654,7 @@
         <v>81</v>
       </c>
       <c r="AO180" t="s" s="2">
-        <v>133</v>
+        <v>81</v>
       </c>
       <c r="AP180" t="s" s="2">
         <v>81</v>
@@ -24649,21 +24665,23 @@
     </row>
     <row r="181" hidden="true">
       <c r="A181" t="s" s="2">
-        <v>671</v>
+        <v>664</v>
       </c>
       <c r="B181" t="s" s="2">
-        <v>672</v>
-      </c>
-      <c r="C181" s="2"/>
+        <v>663</v>
+      </c>
+      <c r="C181" t="s" s="2">
+        <v>665</v>
+      </c>
       <c r="D181" t="s" s="2">
-        <v>81</v>
+        <v>666</v>
       </c>
       <c r="E181" s="2"/>
       <c r="F181" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="G181" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H181" t="s" s="2">
         <v>81</v>
@@ -24675,13 +24693,13 @@
         <v>81</v>
       </c>
       <c r="K181" t="s" s="2">
-        <v>199</v>
+        <v>178</v>
       </c>
       <c r="L181" t="s" s="2">
-        <v>200</v>
+        <v>667</v>
       </c>
       <c r="M181" t="s" s="2">
-        <v>201</v>
+        <v>668</v>
       </c>
       <c r="N181" s="2"/>
       <c r="O181" s="2"/>
@@ -24720,29 +24738,31 @@
         <v>81</v>
       </c>
       <c r="AB181" t="s" s="2">
-        <v>202</v>
-      </c>
-      <c r="AC181" s="2"/>
+        <v>81</v>
+      </c>
+      <c r="AC181" t="s" s="2">
+        <v>81</v>
+      </c>
       <c r="AD181" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE181" t="s" s="2">
-        <v>203</v>
+        <v>81</v>
       </c>
       <c r="AF181" t="s" s="2">
-        <v>204</v>
+        <v>174</v>
       </c>
       <c r="AG181" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH181" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AI181" t="s" s="2">
-        <v>81</v>
+        <v>180</v>
       </c>
       <c r="AJ181" t="s" s="2">
-        <v>81</v>
+        <v>181</v>
       </c>
       <c r="AK181" t="s" s="2">
         <v>81</v>
@@ -24757,7 +24777,7 @@
         <v>81</v>
       </c>
       <c r="AO181" t="s" s="2">
-        <v>133</v>
+        <v>81</v>
       </c>
       <c r="AP181" t="s" s="2">
         <v>81</v>
@@ -24768,20 +24788,18 @@
     </row>
     <row r="182" hidden="true">
       <c r="A182" t="s" s="2">
-        <v>673</v>
+        <v>669</v>
       </c>
       <c r="B182" t="s" s="2">
-        <v>672</v>
-      </c>
-      <c r="C182" t="s" s="2">
-        <v>206</v>
-      </c>
+        <v>670</v>
+      </c>
+      <c r="C182" s="2"/>
       <c r="D182" t="s" s="2">
         <v>81</v>
       </c>
       <c r="E182" s="2"/>
       <c r="F182" t="s" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="G182" t="s" s="2">
         <v>90</v>
@@ -24796,13 +24814,13 @@
         <v>81</v>
       </c>
       <c r="K182" t="s" s="2">
-        <v>199</v>
+        <v>165</v>
       </c>
       <c r="L182" t="s" s="2">
-        <v>200</v>
+        <v>166</v>
       </c>
       <c r="M182" t="s" s="2">
-        <v>201</v>
+        <v>184</v>
       </c>
       <c r="N182" s="2"/>
       <c r="O182" s="2"/>
@@ -24829,13 +24847,13 @@
         <v>81</v>
       </c>
       <c r="X182" t="s" s="2">
-        <v>113</v>
+        <v>81</v>
       </c>
       <c r="Y182" t="s" s="2">
-        <v>674</v>
+        <v>81</v>
       </c>
       <c r="Z182" t="s" s="2">
-        <v>675</v>
+        <v>81</v>
       </c>
       <c r="AA182" t="s" s="2">
         <v>81</v>
@@ -24853,7 +24871,7 @@
         <v>81</v>
       </c>
       <c r="AF182" t="s" s="2">
-        <v>204</v>
+        <v>168</v>
       </c>
       <c r="AG182" t="s" s="2">
         <v>79</v>
@@ -24868,19 +24886,19 @@
         <v>81</v>
       </c>
       <c r="AK182" t="s" s="2">
-        <v>657</v>
+        <v>81</v>
       </c>
       <c r="AL182" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM182" t="s" s="2">
-        <v>657</v>
+        <v>81</v>
       </c>
       <c r="AN182" t="s" s="2">
-        <v>657</v>
+        <v>81</v>
       </c>
       <c r="AO182" t="s" s="2">
-        <v>133</v>
+        <v>185</v>
       </c>
       <c r="AP182" t="s" s="2">
         <v>81</v>
@@ -24891,21 +24909,21 @@
     </row>
     <row r="183" hidden="true">
       <c r="A183" t="s" s="2">
-        <v>676</v>
+        <v>671</v>
       </c>
       <c r="B183" t="s" s="2">
-        <v>676</v>
+        <v>672</v>
       </c>
       <c r="C183" s="2"/>
       <c r="D183" t="s" s="2">
-        <v>81</v>
+        <v>135</v>
       </c>
       <c r="E183" s="2"/>
       <c r="F183" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G183" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H183" t="s" s="2">
         <v>81</v>
@@ -24917,15 +24935,17 @@
         <v>81</v>
       </c>
       <c r="K183" t="s" s="2">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="L183" t="s" s="2">
-        <v>209</v>
+        <v>137</v>
       </c>
       <c r="M183" t="s" s="2">
-        <v>209</v>
-      </c>
-      <c r="N183" s="2"/>
+        <v>188</v>
+      </c>
+      <c r="N183" t="s" s="2">
+        <v>139</v>
+      </c>
       <c r="O183" s="2"/>
       <c r="P183" t="s" s="2">
         <v>81</v>
@@ -24962,25 +24982,25 @@
         <v>81</v>
       </c>
       <c r="AB183" t="s" s="2">
-        <v>81</v>
+        <v>172</v>
       </c>
       <c r="AC183" t="s" s="2">
-        <v>81</v>
+        <v>189</v>
       </c>
       <c r="AD183" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE183" t="s" s="2">
-        <v>81</v>
+        <v>173</v>
       </c>
       <c r="AF183" t="s" s="2">
-        <v>210</v>
+        <v>174</v>
       </c>
       <c r="AG183" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH183" t="s" s="2">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="AI183" t="s" s="2">
         <v>81</v>
@@ -25001,7 +25021,7 @@
         <v>81</v>
       </c>
       <c r="AO183" t="s" s="2">
-        <v>81</v>
+        <v>185</v>
       </c>
       <c r="AP183" t="s" s="2">
         <v>81</v>
@@ -25012,18 +25032,18 @@
     </row>
     <row r="184" hidden="true">
       <c r="A184" t="s" s="2">
-        <v>677</v>
+        <v>673</v>
       </c>
       <c r="B184" t="s" s="2">
-        <v>677</v>
+        <v>674</v>
       </c>
       <c r="C184" s="2"/>
       <c r="D184" t="s" s="2">
-        <v>678</v>
+        <v>81</v>
       </c>
       <c r="E184" s="2"/>
       <c r="F184" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="G184" t="s" s="2">
         <v>90</v>
@@ -25038,16 +25058,16 @@
         <v>81</v>
       </c>
       <c r="K184" t="s" s="2">
-        <v>199</v>
+        <v>103</v>
       </c>
       <c r="L184" t="s" s="2">
-        <v>679</v>
+        <v>192</v>
       </c>
       <c r="M184" t="s" s="2">
-        <v>680</v>
+        <v>193</v>
       </c>
       <c r="N184" t="s" s="2">
-        <v>681</v>
+        <v>194</v>
       </c>
       <c r="O184" s="2"/>
       <c r="P184" t="s" s="2">
@@ -25055,7 +25075,7 @@
       </c>
       <c r="Q184" s="2"/>
       <c r="R184" t="s" s="2">
-        <v>81</v>
+        <v>195</v>
       </c>
       <c r="S184" t="s" s="2">
         <v>81</v>
@@ -25073,11 +25093,13 @@
         <v>81</v>
       </c>
       <c r="X184" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="Y184" s="2"/>
+        <v>81</v>
+      </c>
+      <c r="Y184" t="s" s="2">
+        <v>81</v>
+      </c>
       <c r="Z184" t="s" s="2">
-        <v>682</v>
+        <v>81</v>
       </c>
       <c r="AA184" t="s" s="2">
         <v>81</v>
@@ -25095,10 +25117,10 @@
         <v>81</v>
       </c>
       <c r="AF184" t="s" s="2">
-        <v>677</v>
+        <v>196</v>
       </c>
       <c r="AG184" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="AH184" t="s" s="2">
         <v>90</v>
@@ -25110,19 +25132,19 @@
         <v>81</v>
       </c>
       <c r="AK184" t="s" s="2">
-        <v>683</v>
+        <v>81</v>
       </c>
       <c r="AL184" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AM184" t="s" s="2">
-        <v>683</v>
+        <v>81</v>
       </c>
       <c r="AN184" t="s" s="2">
-        <v>683</v>
+        <v>81</v>
       </c>
       <c r="AO184" t="s" s="2">
-        <v>684</v>
+        <v>133</v>
       </c>
       <c r="AP184" t="s" s="2">
         <v>81</v>
@@ -25133,10 +25155,10 @@
     </row>
     <row r="185" hidden="true">
       <c r="A185" t="s" s="2">
-        <v>685</v>
+        <v>675</v>
       </c>
       <c r="B185" t="s" s="2">
-        <v>685</v>
+        <v>676</v>
       </c>
       <c r="C185" s="2"/>
       <c r="D185" t="s" s="2">
@@ -25144,10 +25166,10 @@
       </c>
       <c r="E185" s="2"/>
       <c r="F185" t="s" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="G185" t="s" s="2">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H185" t="s" s="2">
         <v>81</v>
@@ -25159,17 +25181,15 @@
         <v>81</v>
       </c>
       <c r="K185" t="s" s="2">
-        <v>499</v>
+        <v>199</v>
       </c>
       <c r="L185" t="s" s="2">
-        <v>686</v>
+        <v>200</v>
       </c>
       <c r="M185" t="s" s="2">
-        <v>687</v>
-      </c>
-      <c r="N185" t="s" s="2">
-        <v>688</v>
-      </c>
+        <v>201</v>
+      </c>
+      <c r="N185" s="2"/>
       <c r="O185" s="2"/>
       <c r="P185" t="s" s="2">
         <v>81</v>
@@ -25206,56 +25226,542 @@
         <v>81</v>
       </c>
       <c r="AB185" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AC185" t="s" s="2">
-        <v>81</v>
-      </c>
+        <v>202</v>
+      </c>
+      <c r="AC185" s="2"/>
       <c r="AD185" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AE185" t="s" s="2">
-        <v>81</v>
+        <v>203</v>
       </c>
       <c r="AF185" t="s" s="2">
+        <v>204</v>
+      </c>
+      <c r="AG185" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH185" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI185" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ185" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK185" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL185" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM185" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN185" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO185" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="AP185" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AQ185" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="186" hidden="true">
+      <c r="A186" t="s" s="2">
+        <v>677</v>
+      </c>
+      <c r="B186" t="s" s="2">
+        <v>676</v>
+      </c>
+      <c r="C186" t="s" s="2">
+        <v>206</v>
+      </c>
+      <c r="D186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E186" s="2"/>
+      <c r="F186" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="G186" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="K186" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="L186" t="s" s="2">
+        <v>200</v>
+      </c>
+      <c r="M186" t="s" s="2">
+        <v>201</v>
+      </c>
+      <c r="N186" s="2"/>
+      <c r="O186" s="2"/>
+      <c r="P186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q186" s="2"/>
+      <c r="R186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X186" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="Y186" t="s" s="2">
+        <v>678</v>
+      </c>
+      <c r="Z186" t="s" s="2">
+        <v>679</v>
+      </c>
+      <c r="AA186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF186" t="s" s="2">
+        <v>204</v>
+      </c>
+      <c r="AG186" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH186" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK186" t="s" s="2">
+        <v>661</v>
+      </c>
+      <c r="AL186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM186" t="s" s="2">
+        <v>661</v>
+      </c>
+      <c r="AN186" t="s" s="2">
+        <v>661</v>
+      </c>
+      <c r="AO186" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="AP186" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AQ186" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="187" hidden="true">
+      <c r="A187" t="s" s="2">
+        <v>680</v>
+      </c>
+      <c r="B187" t="s" s="2">
+        <v>680</v>
+      </c>
+      <c r="C187" s="2"/>
+      <c r="D187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E187" s="2"/>
+      <c r="F187" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G187" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="K187" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="L187" t="s" s="2">
+        <v>209</v>
+      </c>
+      <c r="M187" t="s" s="2">
+        <v>209</v>
+      </c>
+      <c r="N187" s="2"/>
+      <c r="O187" s="2"/>
+      <c r="P187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q187" s="2"/>
+      <c r="R187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF187" t="s" s="2">
+        <v>210</v>
+      </c>
+      <c r="AG187" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH187" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AP187" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AQ187" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="188" hidden="true">
+      <c r="A188" t="s" s="2">
+        <v>681</v>
+      </c>
+      <c r="B188" t="s" s="2">
+        <v>681</v>
+      </c>
+      <c r="C188" s="2"/>
+      <c r="D188" t="s" s="2">
+        <v>682</v>
+      </c>
+      <c r="E188" s="2"/>
+      <c r="F188" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G188" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="H188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="K188" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="L188" t="s" s="2">
+        <v>683</v>
+      </c>
+      <c r="M188" t="s" s="2">
+        <v>684</v>
+      </c>
+      <c r="N188" t="s" s="2">
         <v>685</v>
       </c>
-      <c r="AG185" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH185" t="s" s="2">
+      <c r="O188" s="2"/>
+      <c r="P188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q188" s="2"/>
+      <c r="R188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X188" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="Y188" s="2"/>
+      <c r="Z188" t="s" s="2">
+        <v>686</v>
+      </c>
+      <c r="AA188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF188" t="s" s="2">
+        <v>681</v>
+      </c>
+      <c r="AG188" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH188" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="AI188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK188" t="s" s="2">
+        <v>687</v>
+      </c>
+      <c r="AL188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM188" t="s" s="2">
+        <v>687</v>
+      </c>
+      <c r="AN188" t="s" s="2">
+        <v>687</v>
+      </c>
+      <c r="AO188" t="s" s="2">
+        <v>688</v>
+      </c>
+      <c r="AP188" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AQ188" t="s" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="189" hidden="true">
+      <c r="A189" t="s" s="2">
+        <v>689</v>
+      </c>
+      <c r="B189" t="s" s="2">
+        <v>689</v>
+      </c>
+      <c r="C189" s="2"/>
+      <c r="D189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="E189" s="2"/>
+      <c r="F189" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G189" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="AI185" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AJ185" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AK185" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AL185" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AM185" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN185" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AO185" t="s" s="2">
+      <c r="H189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="I189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="J189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="K189" t="s" s="2">
+        <v>499</v>
+      </c>
+      <c r="L189" t="s" s="2">
+        <v>690</v>
+      </c>
+      <c r="M189" t="s" s="2">
+        <v>691</v>
+      </c>
+      <c r="N189" t="s" s="2">
+        <v>692</v>
+      </c>
+      <c r="O189" s="2"/>
+      <c r="P189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Q189" s="2"/>
+      <c r="R189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="S189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="T189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="U189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="V189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="W189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="X189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Y189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="Z189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AA189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AB189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AC189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AD189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AE189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AF189" t="s" s="2">
+        <v>689</v>
+      </c>
+      <c r="AG189" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH189" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AI189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AJ189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AK189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AL189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AM189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AO189" t="s" s="2">
         <v>503</v>
       </c>
-      <c r="AP185" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AQ185" t="s" s="2">
+      <c r="AP189" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AQ189" t="s" s="2">
         <v>81</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AQ185">
+  <autoFilter ref="A1:AQ189">
     <filterColumn colId="6">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -25265,7 +25771,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI184">
+  <conditionalFormatting sqref="A2:AI188">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@e4f0f4295231327c177e630671272f3d02239103 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-AllergyIntolerance.xlsx
+++ b/StructureDefinition-AllergyIntolerance.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-03T11:19:03+00:00</t>
+    <t>2025-02-03T16:53:34+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -510,7 +510,7 @@
     <t>The clinical status of the allergy or intolerance.</t>
   </si>
   <si>
-    <t>This element is labeled as a modifier because the status contains the codes inactive and resolved that mark the AllergyIntolerance as not currently valid.</t>
+    <t>Zie voor mappings [AllergieStatusCodelijst-to-allergy-status](https://simplifier.net/packages/nictiz.fhir.nl.stu3.zib2017/2.2.18/files/2316940)</t>
   </si>
   <si>
     <t>required</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@4af1690b2eea61c78e1da6ba5e6308639471dba6 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-AllergyIntolerance.xlsx
+++ b/StructureDefinition-AllergyIntolerance.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-04T12:12:36+00:00</t>
+    <t>2025-02-05T13:44:35+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -16565,7 +16565,7 @@
         <v>81</v>
       </c>
       <c r="H115" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="I115" t="s" s="2">
         <v>82</v>
@@ -18154,7 +18154,7 @@
         <v>91</v>
       </c>
       <c r="H128" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="I128" t="s" s="2">
         <v>82</v>

</xml_diff>